<commit_message>
feat: add persistent factory data and classified documents
</commit_message>
<xml_diff>
--- a/demo_factory/documents/internal/Station_Layout.xlsx
+++ b/demo_factory/documents/internal/Station_Layout.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FACTORY-DEMO-01" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stations" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,42 +418,358 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Document ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SL-211</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Station Layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Factory</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FACTORY-DEMO-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Revision</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Effective Date</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Demo Operations Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>station_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Station Layout</t>
+          <t>station_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>upstream</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>downstream</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>primary_equipment</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>safety_zone</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>nominal_cycle_time_s</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>owner</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S01 Material Intake through S05 Packaging</t>
+          <t>Material Intake</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Feeder</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SZ-01</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>24</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Material Operations</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Synthetic training data only</t>
+          <t>Positioning</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Positioning fixture</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SZ-02</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>31</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Assembly Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Robot Assembly</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Demo robot</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SZ-03</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>42</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Automation Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Quality Inspection</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Inspection frame</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SZ-04</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>28</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Quality Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Packing cell</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SZ-05</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Packaging Operations</t>
         </is>
       </c>
     </row>

</xml_diff>